<commit_message>
Actualizar RECAUDO_PF.xlsx - 07-05-2026, 4:30:53 p. m.
</commit_message>
<xml_diff>
--- a/data/RECAUDO_PF.xlsx
+++ b/data/RECAUDO_PF.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://funerariaimchile.sharepoint.com/sites/CARTERAVALLESUNIDOS/Shared Documents/Cobranza/2025/MAYO 2026/07-05-2026/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6423BB15-1D83-47ED-935B-6BFBBD651171}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{3E5764EE-C2BF-4006-8DA4-74CA9B7C36A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7068" uniqueCount="1190">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7586" uniqueCount="1277">
   <si>
     <t>EMPRESA</t>
   </si>
@@ -3590,6 +3590,267 @@
   </si>
   <si>
     <t>954061656</t>
+  </si>
+  <si>
+    <t>09/03/2026</t>
+  </si>
+  <si>
+    <t>17241987-9</t>
+  </si>
+  <si>
+    <t>SALINAS SALINAS CAMILO ANDRES</t>
+  </si>
+  <si>
+    <t>camilo.salinas89@gmail.com</t>
+  </si>
+  <si>
+    <t>949508704</t>
+  </si>
+  <si>
+    <t>07/02/2025</t>
+  </si>
+  <si>
+    <t>10693767-2</t>
+  </si>
+  <si>
+    <t>PACHECO VIVEROS LETICIA SOLEDAD</t>
+  </si>
+  <si>
+    <t>Vitacura</t>
+  </si>
+  <si>
+    <t>leticiapachecoviveros@gmail.com</t>
+  </si>
+  <si>
+    <t>965896509</t>
+  </si>
+  <si>
+    <t>994329189</t>
+  </si>
+  <si>
+    <t>06/01/2026</t>
+  </si>
+  <si>
+    <t>10706660-8</t>
+  </si>
+  <si>
+    <t>CARTER GONZALES ROBERTO GERMAN</t>
+  </si>
+  <si>
+    <t>roberto.carter@grupocerromoreno.cl</t>
+  </si>
+  <si>
+    <t>979988262</t>
+  </si>
+  <si>
+    <t>14/10/2025</t>
+  </si>
+  <si>
+    <t>5351195-3</t>
+  </si>
+  <si>
+    <t>VALDES INOSTROZA ESTANISLAO DEL CARMEN</t>
+  </si>
+  <si>
+    <t>tanyvaldesinostroza@gmail.com</t>
+  </si>
+  <si>
+    <t>993323212</t>
+  </si>
+  <si>
+    <t>12/05/2025</t>
+  </si>
+  <si>
+    <t>10506783-6</t>
+  </si>
+  <si>
+    <t>GARRIDO MERA SANDRA DEL ROSARIO</t>
+  </si>
+  <si>
+    <t>sandragarridomera12@gmail.com</t>
+  </si>
+  <si>
+    <t>988114795</t>
+  </si>
+  <si>
+    <t>12879044-6</t>
+  </si>
+  <si>
+    <t>ACOSTA PINO VERÓNICA FLORENTICA</t>
+  </si>
+  <si>
+    <t>zoeclo46@gmail.com</t>
+  </si>
+  <si>
+    <t>959079259</t>
+  </si>
+  <si>
+    <t>ANA ROSA BURBOA FERNANDEZ</t>
+  </si>
+  <si>
+    <t>24/12/2024</t>
+  </si>
+  <si>
+    <t>12668958-6</t>
+  </si>
+  <si>
+    <t>GONZALEZ MUÑOZ JENNY ANDREA</t>
+  </si>
+  <si>
+    <t>jenny.gonzalez01936@gmail.com</t>
+  </si>
+  <si>
+    <t>984060823</t>
+  </si>
+  <si>
+    <t>8116330-8</t>
+  </si>
+  <si>
+    <t>GUERRA ZAGAL CECILIA ANGELICA</t>
+  </si>
+  <si>
+    <t>San Ramón</t>
+  </si>
+  <si>
+    <t>angelicaguerra4059@gmail.com</t>
+  </si>
+  <si>
+    <t>993615020</t>
+  </si>
+  <si>
+    <t>7896837-0</t>
+  </si>
+  <si>
+    <t>MUÑOZ SALAZAR ROSA ADELAIDA</t>
+  </si>
+  <si>
+    <t>RRojas</t>
+  </si>
+  <si>
+    <t>rosaadelaida1957@gmail.com</t>
+  </si>
+  <si>
+    <t>950980306</t>
+  </si>
+  <si>
+    <t>05/12/2025</t>
+  </si>
+  <si>
+    <t>10947894-6</t>
+  </si>
+  <si>
+    <t>IBARRA PAILLAO MARIA LILIANA</t>
+  </si>
+  <si>
+    <t>Mlilybarra@gmail.com</t>
+  </si>
+  <si>
+    <t>990877741</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Emperatriz Alexandra Franco Mosquera </t>
+  </si>
+  <si>
+    <t>10882279-1</t>
+  </si>
+  <si>
+    <t>BADILLA PAREDES JOSE RIGOBERTO</t>
+  </si>
+  <si>
+    <t>26325144-8</t>
+  </si>
+  <si>
+    <t>clascondes</t>
+  </si>
+  <si>
+    <t>HASTA 60 D</t>
+  </si>
+  <si>
+    <t>jobadilla1966@gmail.com</t>
+  </si>
+  <si>
+    <t>953659587</t>
+  </si>
+  <si>
+    <t>7849847-1</t>
+  </si>
+  <si>
+    <t>GALVEZ VARGAS ALICIA DEDEL CARMEN</t>
+  </si>
+  <si>
+    <t>aliciagalvezv@gmail.com</t>
+  </si>
+  <si>
+    <t>942097690</t>
+  </si>
+  <si>
+    <t>931306476</t>
+  </si>
+  <si>
+    <t>ANGELICA MARIA MUÑOZ YAÑEZ</t>
+  </si>
+  <si>
+    <t>07/11/2024</t>
+  </si>
+  <si>
+    <t>9625116-5</t>
+  </si>
+  <si>
+    <t>MORENO MIRANDA MARISOL DEL CARMEN</t>
+  </si>
+  <si>
+    <t>MARISOLCARMENMORENO@GMAIL.COM</t>
+  </si>
+  <si>
+    <t>989244061</t>
+  </si>
+  <si>
+    <t>6389577-6</t>
+  </si>
+  <si>
+    <t>MARTINEZ MIRANDA VICTORIA DE LAS MERCEDES</t>
+  </si>
+  <si>
+    <t>VICTORIAMIRANDA73MARTINEZ@GMAIL.COM</t>
+  </si>
+  <si>
+    <t>968401212</t>
+  </si>
+  <si>
+    <t>RICARDO JAVIER NAIPIL BURGOS</t>
+  </si>
+  <si>
+    <t>11650516-9</t>
+  </si>
+  <si>
+    <t>RODRIGUEZ CACERES EUGENIA DE LAS MERCEDES</t>
+  </si>
+  <si>
+    <t>kenita.rodriguez70@gmail.com</t>
+  </si>
+  <si>
+    <t>990032443</t>
+  </si>
+  <si>
+    <t xml:space="preserve">María Isabel Gutiérrez  </t>
+  </si>
+  <si>
+    <t>20/03/2026</t>
+  </si>
+  <si>
+    <t>19936540-1</t>
+  </si>
+  <si>
+    <t>ARZOLA GUTIERREZ MARÍA JOSE</t>
+  </si>
+  <si>
+    <t>kote27.arzola@hotmail.com</t>
+  </si>
+  <si>
+    <t>932405178</t>
+  </si>
+  <si>
+    <t>988044270</t>
   </si>
 </sst>
 </file>
@@ -3966,7 +4227,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AV258"/>
+  <dimension ref="A1:AV277"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="25.796875" customWidth="1"/>
@@ -38034,10 +38295,2514 @@
         <v>1189</v>
       </c>
     </row>
+    <row r="259" spans="1:48" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A259" t="s">
+        <v>48</v>
+      </c>
+      <c r="B259" t="s">
+        <v>138</v>
+      </c>
+      <c r="C259" t="s">
+        <v>1190</v>
+      </c>
+      <c r="D259" t="s">
+        <v>1191</v>
+      </c>
+      <c r="E259" t="s">
+        <v>1192</v>
+      </c>
+      <c r="F259" t="s">
+        <v>53</v>
+      </c>
+      <c r="G259" t="s">
+        <v>111</v>
+      </c>
+      <c r="H259" t="s">
+        <v>55</v>
+      </c>
+      <c r="I259">
+        <v>3832</v>
+      </c>
+      <c r="J259" t="s">
+        <v>56</v>
+      </c>
+      <c r="K259">
+        <v>53438</v>
+      </c>
+      <c r="L259">
+        <v>53438</v>
+      </c>
+      <c r="M259">
+        <v>48</v>
+      </c>
+      <c r="N259">
+        <v>7</v>
+      </c>
+      <c r="O259" t="s">
+        <v>1178</v>
+      </c>
+      <c r="P259">
+        <v>53438</v>
+      </c>
+      <c r="Q259">
+        <v>53438</v>
+      </c>
+      <c r="R259" t="s">
+        <v>58</v>
+      </c>
+      <c r="S259">
+        <v>46</v>
+      </c>
+      <c r="T259">
+        <v>1</v>
+      </c>
+      <c r="U259">
+        <v>1</v>
+      </c>
+      <c r="V259">
+        <v>1</v>
+      </c>
+      <c r="W259" t="s">
+        <v>59</v>
+      </c>
+      <c r="X259" t="s">
+        <v>60</v>
+      </c>
+      <c r="Y259" t="s">
+        <v>61</v>
+      </c>
+      <c r="Z259" t="s">
+        <v>62</v>
+      </c>
+      <c r="AA259" t="s">
+        <v>62</v>
+      </c>
+      <c r="AB259" t="s">
+        <v>58</v>
+      </c>
+      <c r="AD259" t="s">
+        <v>62</v>
+      </c>
+      <c r="AE259" t="s">
+        <v>58</v>
+      </c>
+      <c r="AF259" t="s">
+        <v>63</v>
+      </c>
+      <c r="AG259">
+        <v>-31</v>
+      </c>
+      <c r="AH259">
+        <v>0</v>
+      </c>
+      <c r="AI259">
+        <v>0</v>
+      </c>
+      <c r="AJ259" t="s">
+        <v>64</v>
+      </c>
+      <c r="AK259" t="s">
+        <v>65</v>
+      </c>
+      <c r="AL259" t="s">
+        <v>66</v>
+      </c>
+      <c r="AM259">
+        <v>971855</v>
+      </c>
+      <c r="AN259">
+        <v>135171</v>
+      </c>
+      <c r="AS259" t="s">
+        <v>85</v>
+      </c>
+      <c r="AT259" t="s">
+        <v>1193</v>
+      </c>
+      <c r="AV259" t="s">
+        <v>1194</v>
+      </c>
+    </row>
+    <row r="260" spans="1:48" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A260" t="s">
+        <v>48</v>
+      </c>
+      <c r="B260" t="s">
+        <v>323</v>
+      </c>
+      <c r="C260" t="s">
+        <v>1195</v>
+      </c>
+      <c r="D260" t="s">
+        <v>1196</v>
+      </c>
+      <c r="E260" t="s">
+        <v>1197</v>
+      </c>
+      <c r="F260" t="s">
+        <v>53</v>
+      </c>
+      <c r="G260" t="s">
+        <v>1198</v>
+      </c>
+      <c r="H260" t="s">
+        <v>104</v>
+      </c>
+      <c r="I260">
+        <v>565</v>
+      </c>
+      <c r="J260" t="s">
+        <v>56</v>
+      </c>
+      <c r="K260">
+        <v>40000</v>
+      </c>
+      <c r="L260">
+        <v>40000</v>
+      </c>
+      <c r="M260">
+        <v>36</v>
+      </c>
+      <c r="N260">
+        <v>7</v>
+      </c>
+      <c r="O260" t="s">
+        <v>1178</v>
+      </c>
+      <c r="P260">
+        <v>40000</v>
+      </c>
+      <c r="Q260">
+        <v>40000</v>
+      </c>
+      <c r="R260" t="s">
+        <v>58</v>
+      </c>
+      <c r="S260">
+        <v>21</v>
+      </c>
+      <c r="T260">
+        <v>15</v>
+      </c>
+      <c r="U260">
+        <v>1</v>
+      </c>
+      <c r="V260">
+        <v>15</v>
+      </c>
+      <c r="W260" t="s">
+        <v>59</v>
+      </c>
+      <c r="X260" t="s">
+        <v>60</v>
+      </c>
+      <c r="Y260" t="s">
+        <v>61</v>
+      </c>
+      <c r="Z260" t="s">
+        <v>62</v>
+      </c>
+      <c r="AA260" t="s">
+        <v>62</v>
+      </c>
+      <c r="AB260" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC260" t="s">
+        <v>95</v>
+      </c>
+      <c r="AD260" t="s">
+        <v>62</v>
+      </c>
+      <c r="AE260" t="s">
+        <v>58</v>
+      </c>
+      <c r="AF260" t="s">
+        <v>63</v>
+      </c>
+      <c r="AG260">
+        <v>-31</v>
+      </c>
+      <c r="AH260">
+        <v>0</v>
+      </c>
+      <c r="AI260">
+        <v>0</v>
+      </c>
+      <c r="AJ260" t="s">
+        <v>64</v>
+      </c>
+      <c r="AK260" t="s">
+        <v>65</v>
+      </c>
+      <c r="AL260" t="s">
+        <v>66</v>
+      </c>
+      <c r="AM260">
+        <v>971856</v>
+      </c>
+      <c r="AN260">
+        <v>133446</v>
+      </c>
+      <c r="AS260" t="s">
+        <v>77</v>
+      </c>
+      <c r="AT260" t="s">
+        <v>1199</v>
+      </c>
+      <c r="AU260" t="s">
+        <v>1200</v>
+      </c>
+      <c r="AV260" t="s">
+        <v>1201</v>
+      </c>
+    </row>
+    <row r="261" spans="1:48" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A261" t="s">
+        <v>48</v>
+      </c>
+      <c r="B261" t="s">
+        <v>504</v>
+      </c>
+      <c r="C261" t="s">
+        <v>1202</v>
+      </c>
+      <c r="D261" t="s">
+        <v>1203</v>
+      </c>
+      <c r="E261" t="s">
+        <v>1204</v>
+      </c>
+      <c r="F261" t="s">
+        <v>53</v>
+      </c>
+      <c r="G261" t="s">
+        <v>111</v>
+      </c>
+      <c r="H261" t="s">
+        <v>55</v>
+      </c>
+      <c r="I261">
+        <v>3055</v>
+      </c>
+      <c r="J261" t="s">
+        <v>56</v>
+      </c>
+      <c r="K261">
+        <v>86364</v>
+      </c>
+      <c r="L261">
+        <v>86364</v>
+      </c>
+      <c r="M261">
+        <v>66</v>
+      </c>
+      <c r="N261">
+        <v>7</v>
+      </c>
+      <c r="O261" t="s">
+        <v>1178</v>
+      </c>
+      <c r="P261">
+        <v>86364</v>
+      </c>
+      <c r="Q261">
+        <v>86364</v>
+      </c>
+      <c r="R261" t="s">
+        <v>58</v>
+      </c>
+      <c r="S261">
+        <v>62</v>
+      </c>
+      <c r="T261">
+        <v>4</v>
+      </c>
+      <c r="U261">
+        <v>1</v>
+      </c>
+      <c r="V261">
+        <v>4</v>
+      </c>
+      <c r="W261" t="s">
+        <v>59</v>
+      </c>
+      <c r="X261" t="s">
+        <v>60</v>
+      </c>
+      <c r="Y261" t="s">
+        <v>61</v>
+      </c>
+      <c r="Z261" t="s">
+        <v>62</v>
+      </c>
+      <c r="AA261" t="s">
+        <v>62</v>
+      </c>
+      <c r="AB261" t="s">
+        <v>58</v>
+      </c>
+      <c r="AD261" t="s">
+        <v>62</v>
+      </c>
+      <c r="AE261" t="s">
+        <v>58</v>
+      </c>
+      <c r="AF261" t="s">
+        <v>63</v>
+      </c>
+      <c r="AG261">
+        <v>-31</v>
+      </c>
+      <c r="AH261">
+        <v>0</v>
+      </c>
+      <c r="AI261">
+        <v>0</v>
+      </c>
+      <c r="AJ261" t="s">
+        <v>64</v>
+      </c>
+      <c r="AK261" t="s">
+        <v>65</v>
+      </c>
+      <c r="AL261" t="s">
+        <v>66</v>
+      </c>
+      <c r="AM261">
+        <v>971857</v>
+      </c>
+      <c r="AN261">
+        <v>134957</v>
+      </c>
+      <c r="AS261" t="s">
+        <v>312</v>
+      </c>
+      <c r="AT261" t="s">
+        <v>1205</v>
+      </c>
+      <c r="AU261" t="s">
+        <v>87</v>
+      </c>
+      <c r="AV261" t="s">
+        <v>1206</v>
+      </c>
+    </row>
+    <row r="262" spans="1:48" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A262" t="s">
+        <v>48</v>
+      </c>
+      <c r="B262" t="s">
+        <v>331</v>
+      </c>
+      <c r="C262" t="s">
+        <v>1207</v>
+      </c>
+      <c r="D262" t="s">
+        <v>1208</v>
+      </c>
+      <c r="E262" t="s">
+        <v>1209</v>
+      </c>
+      <c r="F262" t="s">
+        <v>53</v>
+      </c>
+      <c r="G262" t="s">
+        <v>54</v>
+      </c>
+      <c r="H262" t="s">
+        <v>55</v>
+      </c>
+      <c r="I262">
+        <v>1908</v>
+      </c>
+      <c r="J262" t="s">
+        <v>56</v>
+      </c>
+      <c r="K262">
+        <v>75833</v>
+      </c>
+      <c r="L262">
+        <v>75833</v>
+      </c>
+      <c r="M262">
+        <v>36</v>
+      </c>
+      <c r="N262">
+        <v>23</v>
+      </c>
+      <c r="O262" t="s">
+        <v>1178</v>
+      </c>
+      <c r="P262">
+        <v>75833</v>
+      </c>
+      <c r="Q262">
+        <v>75833</v>
+      </c>
+      <c r="R262" t="s">
+        <v>58</v>
+      </c>
+      <c r="S262">
+        <v>26</v>
+      </c>
+      <c r="T262">
+        <v>10</v>
+      </c>
+      <c r="U262">
+        <v>1</v>
+      </c>
+      <c r="V262">
+        <v>9</v>
+      </c>
+      <c r="W262" t="s">
+        <v>59</v>
+      </c>
+      <c r="X262" t="s">
+        <v>210</v>
+      </c>
+      <c r="Y262" t="s">
+        <v>61</v>
+      </c>
+      <c r="Z262" t="s">
+        <v>425</v>
+      </c>
+      <c r="AA262" t="s">
+        <v>425</v>
+      </c>
+      <c r="AB262" t="s">
+        <v>58</v>
+      </c>
+      <c r="AD262" t="s">
+        <v>426</v>
+      </c>
+      <c r="AE262" t="s">
+        <v>58</v>
+      </c>
+      <c r="AF262" t="s">
+        <v>63</v>
+      </c>
+      <c r="AG262">
+        <v>-139</v>
+      </c>
+      <c r="AH262">
+        <v>0</v>
+      </c>
+      <c r="AI262">
+        <v>0</v>
+      </c>
+      <c r="AJ262" t="s">
+        <v>64</v>
+      </c>
+      <c r="AK262" t="s">
+        <v>65</v>
+      </c>
+      <c r="AL262" t="s">
+        <v>66</v>
+      </c>
+      <c r="AM262">
+        <v>971859</v>
+      </c>
+      <c r="AN262">
+        <v>134599</v>
+      </c>
+      <c r="AS262" t="s">
+        <v>268</v>
+      </c>
+      <c r="AT262" t="s">
+        <v>1210</v>
+      </c>
+      <c r="AU262" t="s">
+        <v>87</v>
+      </c>
+      <c r="AV262" t="s">
+        <v>1211</v>
+      </c>
+    </row>
+    <row r="263" spans="1:48" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A263" t="s">
+        <v>48</v>
+      </c>
+      <c r="B263" t="s">
+        <v>331</v>
+      </c>
+      <c r="C263" t="s">
+        <v>1207</v>
+      </c>
+      <c r="D263" t="s">
+        <v>1208</v>
+      </c>
+      <c r="E263" t="s">
+        <v>1209</v>
+      </c>
+      <c r="F263" t="s">
+        <v>53</v>
+      </c>
+      <c r="G263" t="s">
+        <v>54</v>
+      </c>
+      <c r="H263" t="s">
+        <v>55</v>
+      </c>
+      <c r="I263">
+        <v>1908</v>
+      </c>
+      <c r="J263" t="s">
+        <v>56</v>
+      </c>
+      <c r="K263">
+        <v>75833</v>
+      </c>
+      <c r="L263">
+        <v>75833</v>
+      </c>
+      <c r="M263">
+        <v>36</v>
+      </c>
+      <c r="N263">
+        <v>23</v>
+      </c>
+      <c r="O263" t="s">
+        <v>1178</v>
+      </c>
+      <c r="P263">
+        <v>75833</v>
+      </c>
+      <c r="Q263">
+        <v>75833</v>
+      </c>
+      <c r="R263" t="s">
+        <v>58</v>
+      </c>
+      <c r="S263">
+        <v>26</v>
+      </c>
+      <c r="T263">
+        <v>10</v>
+      </c>
+      <c r="U263">
+        <v>1</v>
+      </c>
+      <c r="V263">
+        <v>10</v>
+      </c>
+      <c r="W263" t="s">
+        <v>59</v>
+      </c>
+      <c r="X263" t="s">
+        <v>210</v>
+      </c>
+      <c r="Y263" t="s">
+        <v>61</v>
+      </c>
+      <c r="Z263" t="s">
+        <v>425</v>
+      </c>
+      <c r="AA263" t="s">
+        <v>425</v>
+      </c>
+      <c r="AB263" t="s">
+        <v>58</v>
+      </c>
+      <c r="AD263" t="s">
+        <v>426</v>
+      </c>
+      <c r="AE263" t="s">
+        <v>58</v>
+      </c>
+      <c r="AF263" t="s">
+        <v>63</v>
+      </c>
+      <c r="AG263">
+        <v>-139</v>
+      </c>
+      <c r="AH263">
+        <v>0</v>
+      </c>
+      <c r="AI263">
+        <v>0</v>
+      </c>
+      <c r="AJ263" t="s">
+        <v>64</v>
+      </c>
+      <c r="AK263" t="s">
+        <v>65</v>
+      </c>
+      <c r="AL263" t="s">
+        <v>66</v>
+      </c>
+      <c r="AM263">
+        <v>971859</v>
+      </c>
+      <c r="AN263">
+        <v>134599</v>
+      </c>
+      <c r="AS263" t="s">
+        <v>268</v>
+      </c>
+      <c r="AT263" t="s">
+        <v>1210</v>
+      </c>
+      <c r="AU263" t="s">
+        <v>87</v>
+      </c>
+      <c r="AV263" t="s">
+        <v>1211</v>
+      </c>
+    </row>
+    <row r="264" spans="1:48" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A264" t="s">
+        <v>48</v>
+      </c>
+      <c r="B264" t="s">
+        <v>70</v>
+      </c>
+      <c r="C264" t="s">
+        <v>1212</v>
+      </c>
+      <c r="D264" t="s">
+        <v>1213</v>
+      </c>
+      <c r="E264" t="s">
+        <v>1214</v>
+      </c>
+      <c r="F264" t="s">
+        <v>53</v>
+      </c>
+      <c r="G264" t="s">
+        <v>84</v>
+      </c>
+      <c r="H264" t="s">
+        <v>55</v>
+      </c>
+      <c r="I264">
+        <v>1213</v>
+      </c>
+      <c r="J264" t="s">
+        <v>56</v>
+      </c>
+      <c r="K264">
+        <v>104167</v>
+      </c>
+      <c r="L264">
+        <v>104167</v>
+      </c>
+      <c r="M264">
+        <v>24</v>
+      </c>
+      <c r="N264">
+        <v>8</v>
+      </c>
+      <c r="O264" t="s">
+        <v>1178</v>
+      </c>
+      <c r="P264">
+        <v>104146</v>
+      </c>
+      <c r="Q264">
+        <v>104146</v>
+      </c>
+      <c r="R264" t="s">
+        <v>58</v>
+      </c>
+      <c r="S264">
+        <v>11</v>
+      </c>
+      <c r="T264">
+        <v>14</v>
+      </c>
+      <c r="U264">
+        <v>1</v>
+      </c>
+      <c r="V264">
+        <v>13</v>
+      </c>
+      <c r="W264" t="s">
+        <v>59</v>
+      </c>
+      <c r="X264" t="s">
+        <v>240</v>
+      </c>
+      <c r="Y264" t="s">
+        <v>61</v>
+      </c>
+      <c r="Z264" t="s">
+        <v>550</v>
+      </c>
+      <c r="AA264" t="s">
+        <v>550</v>
+      </c>
+      <c r="AB264" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC264" t="s">
+        <v>76</v>
+      </c>
+      <c r="AD264" t="s">
+        <v>543</v>
+      </c>
+      <c r="AE264" t="s">
+        <v>58</v>
+      </c>
+      <c r="AF264" t="s">
+        <v>63</v>
+      </c>
+      <c r="AG264">
+        <v>-32</v>
+      </c>
+      <c r="AH264">
+        <v>0</v>
+      </c>
+      <c r="AI264">
+        <v>0</v>
+      </c>
+      <c r="AJ264" t="s">
+        <v>64</v>
+      </c>
+      <c r="AK264" t="s">
+        <v>65</v>
+      </c>
+      <c r="AL264" t="s">
+        <v>66</v>
+      </c>
+      <c r="AM264">
+        <v>971861</v>
+      </c>
+      <c r="AN264">
+        <v>134242</v>
+      </c>
+      <c r="AS264" t="s">
+        <v>120</v>
+      </c>
+      <c r="AT264" t="s">
+        <v>1215</v>
+      </c>
+      <c r="AU264" t="s">
+        <v>1216</v>
+      </c>
+      <c r="AV264" t="s">
+        <v>1216</v>
+      </c>
+    </row>
+    <row r="265" spans="1:48" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A265" t="s">
+        <v>48</v>
+      </c>
+      <c r="B265" t="s">
+        <v>70</v>
+      </c>
+      <c r="C265" t="s">
+        <v>1212</v>
+      </c>
+      <c r="D265" t="s">
+        <v>1213</v>
+      </c>
+      <c r="E265" t="s">
+        <v>1214</v>
+      </c>
+      <c r="F265" t="s">
+        <v>53</v>
+      </c>
+      <c r="G265" t="s">
+        <v>84</v>
+      </c>
+      <c r="H265" t="s">
+        <v>55</v>
+      </c>
+      <c r="I265">
+        <v>1213</v>
+      </c>
+      <c r="J265" t="s">
+        <v>56</v>
+      </c>
+      <c r="K265">
+        <v>104167</v>
+      </c>
+      <c r="L265">
+        <v>104167</v>
+      </c>
+      <c r="M265">
+        <v>24</v>
+      </c>
+      <c r="N265">
+        <v>8</v>
+      </c>
+      <c r="O265" t="s">
+        <v>1178</v>
+      </c>
+      <c r="P265">
+        <v>21</v>
+      </c>
+      <c r="Q265">
+        <v>21</v>
+      </c>
+      <c r="R265" t="s">
+        <v>58</v>
+      </c>
+      <c r="S265">
+        <v>11</v>
+      </c>
+      <c r="T265">
+        <v>14</v>
+      </c>
+      <c r="U265">
+        <v>1</v>
+      </c>
+      <c r="V265">
+        <v>14</v>
+      </c>
+      <c r="W265" t="s">
+        <v>59</v>
+      </c>
+      <c r="X265" t="s">
+        <v>240</v>
+      </c>
+      <c r="Y265" t="s">
+        <v>61</v>
+      </c>
+      <c r="Z265" t="s">
+        <v>550</v>
+      </c>
+      <c r="AA265" t="s">
+        <v>550</v>
+      </c>
+      <c r="AB265" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC265" t="s">
+        <v>76</v>
+      </c>
+      <c r="AD265" t="s">
+        <v>543</v>
+      </c>
+      <c r="AE265" t="s">
+        <v>58</v>
+      </c>
+      <c r="AF265" t="s">
+        <v>63</v>
+      </c>
+      <c r="AG265">
+        <v>-32</v>
+      </c>
+      <c r="AH265">
+        <v>0</v>
+      </c>
+      <c r="AI265">
+        <v>0</v>
+      </c>
+      <c r="AJ265" t="s">
+        <v>64</v>
+      </c>
+      <c r="AK265" t="s">
+        <v>65</v>
+      </c>
+      <c r="AL265" t="s">
+        <v>66</v>
+      </c>
+      <c r="AM265">
+        <v>971861</v>
+      </c>
+      <c r="AN265">
+        <v>134242</v>
+      </c>
+      <c r="AS265" t="s">
+        <v>120</v>
+      </c>
+      <c r="AT265" t="s">
+        <v>1215</v>
+      </c>
+      <c r="AU265" t="s">
+        <v>1216</v>
+      </c>
+      <c r="AV265" t="s">
+        <v>1216</v>
+      </c>
+    </row>
+    <row r="266" spans="1:48" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A266" t="s">
+        <v>48</v>
+      </c>
+      <c r="B266" t="s">
+        <v>316</v>
+      </c>
+      <c r="C266" t="s">
+        <v>377</v>
+      </c>
+      <c r="D266" t="s">
+        <v>1217</v>
+      </c>
+      <c r="E266" t="s">
+        <v>1218</v>
+      </c>
+      <c r="F266" t="s">
+        <v>53</v>
+      </c>
+      <c r="G266" t="s">
+        <v>408</v>
+      </c>
+      <c r="H266" t="s">
+        <v>55</v>
+      </c>
+      <c r="I266">
+        <v>2918</v>
+      </c>
+      <c r="J266" t="s">
+        <v>56</v>
+      </c>
+      <c r="K266">
+        <v>25500</v>
+      </c>
+      <c r="L266">
+        <v>25500</v>
+      </c>
+      <c r="M266">
+        <v>60</v>
+      </c>
+      <c r="N266">
+        <v>5</v>
+      </c>
+      <c r="O266" t="s">
+        <v>1178</v>
+      </c>
+      <c r="P266">
+        <v>500</v>
+      </c>
+      <c r="Q266">
+        <v>500</v>
+      </c>
+      <c r="R266" t="s">
+        <v>58</v>
+      </c>
+      <c r="S266">
+        <v>56</v>
+      </c>
+      <c r="T266">
+        <v>4</v>
+      </c>
+      <c r="U266">
+        <v>1</v>
+      </c>
+      <c r="V266">
+        <v>4</v>
+      </c>
+      <c r="W266" t="s">
+        <v>59</v>
+      </c>
+      <c r="X266" t="s">
+        <v>240</v>
+      </c>
+      <c r="Y266" t="s">
+        <v>61</v>
+      </c>
+      <c r="Z266" t="s">
+        <v>550</v>
+      </c>
+      <c r="AA266" t="s">
+        <v>550</v>
+      </c>
+      <c r="AB266" t="s">
+        <v>58</v>
+      </c>
+      <c r="AD266" t="s">
+        <v>543</v>
+      </c>
+      <c r="AE266" t="s">
+        <v>58</v>
+      </c>
+      <c r="AF266" t="s">
+        <v>63</v>
+      </c>
+      <c r="AG266">
+        <v>-29</v>
+      </c>
+      <c r="AH266">
+        <v>7</v>
+      </c>
+      <c r="AI266">
+        <v>0</v>
+      </c>
+      <c r="AJ266" t="s">
+        <v>64</v>
+      </c>
+      <c r="AK266" t="s">
+        <v>65</v>
+      </c>
+      <c r="AL266" t="s">
+        <v>66</v>
+      </c>
+      <c r="AM266">
+        <v>971863</v>
+      </c>
+      <c r="AN266">
+        <v>134905</v>
+      </c>
+      <c r="AS266" t="s">
+        <v>202</v>
+      </c>
+      <c r="AT266" t="s">
+        <v>1219</v>
+      </c>
+      <c r="AU266" t="s">
+        <v>1220</v>
+      </c>
+      <c r="AV266" t="s">
+        <v>1220</v>
+      </c>
+    </row>
+    <row r="267" spans="1:48" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A267" t="s">
+        <v>48</v>
+      </c>
+      <c r="B267" t="s">
+        <v>1221</v>
+      </c>
+      <c r="C267" t="s">
+        <v>1222</v>
+      </c>
+      <c r="D267" t="s">
+        <v>1223</v>
+      </c>
+      <c r="E267" t="s">
+        <v>1224</v>
+      </c>
+      <c r="F267" t="s">
+        <v>53</v>
+      </c>
+      <c r="G267" t="s">
+        <v>209</v>
+      </c>
+      <c r="H267" t="s">
+        <v>104</v>
+      </c>
+      <c r="I267">
+        <v>373</v>
+      </c>
+      <c r="J267" t="s">
+        <v>56</v>
+      </c>
+      <c r="K267">
+        <v>47500</v>
+      </c>
+      <c r="L267">
+        <v>47500</v>
+      </c>
+      <c r="M267">
+        <v>24</v>
+      </c>
+      <c r="N267">
+        <v>6</v>
+      </c>
+      <c r="O267" t="s">
+        <v>1178</v>
+      </c>
+      <c r="P267">
+        <v>47500</v>
+      </c>
+      <c r="Q267">
+        <v>47500</v>
+      </c>
+      <c r="R267" t="s">
+        <v>58</v>
+      </c>
+      <c r="S267">
+        <v>8</v>
+      </c>
+      <c r="T267">
+        <v>16</v>
+      </c>
+      <c r="U267">
+        <v>1</v>
+      </c>
+      <c r="V267">
+        <v>16</v>
+      </c>
+      <c r="W267" t="s">
+        <v>59</v>
+      </c>
+      <c r="X267" t="s">
+        <v>240</v>
+      </c>
+      <c r="Y267" t="s">
+        <v>61</v>
+      </c>
+      <c r="Z267" t="s">
+        <v>550</v>
+      </c>
+      <c r="AA267" t="s">
+        <v>550</v>
+      </c>
+      <c r="AB267" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC267" t="s">
+        <v>95</v>
+      </c>
+      <c r="AD267" t="s">
+        <v>543</v>
+      </c>
+      <c r="AE267" t="s">
+        <v>58</v>
+      </c>
+      <c r="AF267" t="s">
+        <v>63</v>
+      </c>
+      <c r="AG267">
+        <v>-30</v>
+      </c>
+      <c r="AH267">
+        <v>0</v>
+      </c>
+      <c r="AI267">
+        <v>0</v>
+      </c>
+      <c r="AJ267" t="s">
+        <v>64</v>
+      </c>
+      <c r="AK267" t="s">
+        <v>65</v>
+      </c>
+      <c r="AL267" t="s">
+        <v>66</v>
+      </c>
+      <c r="AM267">
+        <v>971865</v>
+      </c>
+      <c r="AN267">
+        <v>133371</v>
+      </c>
+      <c r="AS267" t="s">
+        <v>77</v>
+      </c>
+      <c r="AT267" t="s">
+        <v>1225</v>
+      </c>
+      <c r="AU267" t="s">
+        <v>87</v>
+      </c>
+      <c r="AV267" t="s">
+        <v>1226</v>
+      </c>
+    </row>
+    <row r="268" spans="1:48" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A268" t="s">
+        <v>48</v>
+      </c>
+      <c r="B268" t="s">
+        <v>353</v>
+      </c>
+      <c r="C268" t="s">
+        <v>837</v>
+      </c>
+      <c r="D268" t="s">
+        <v>1227</v>
+      </c>
+      <c r="E268" t="s">
+        <v>1228</v>
+      </c>
+      <c r="F268" t="s">
+        <v>53</v>
+      </c>
+      <c r="G268" t="s">
+        <v>1229</v>
+      </c>
+      <c r="H268" t="s">
+        <v>55</v>
+      </c>
+      <c r="I268">
+        <v>2797</v>
+      </c>
+      <c r="J268" t="s">
+        <v>56</v>
+      </c>
+      <c r="K268">
+        <v>40000</v>
+      </c>
+      <c r="L268">
+        <v>40000</v>
+      </c>
+      <c r="M268">
+        <v>35</v>
+      </c>
+      <c r="N268">
+        <v>30</v>
+      </c>
+      <c r="O268" t="s">
+        <v>1178</v>
+      </c>
+      <c r="P268">
+        <v>40000</v>
+      </c>
+      <c r="Q268">
+        <v>40000</v>
+      </c>
+      <c r="R268" t="s">
+        <v>58</v>
+      </c>
+      <c r="S268">
+        <v>30</v>
+      </c>
+      <c r="T268">
+        <v>5</v>
+      </c>
+      <c r="U268">
+        <v>1</v>
+      </c>
+      <c r="V268">
+        <v>5</v>
+      </c>
+      <c r="W268" t="s">
+        <v>59</v>
+      </c>
+      <c r="X268" t="s">
+        <v>240</v>
+      </c>
+      <c r="Y268" t="s">
+        <v>61</v>
+      </c>
+      <c r="Z268" t="s">
+        <v>550</v>
+      </c>
+      <c r="AA268" t="s">
+        <v>550</v>
+      </c>
+      <c r="AB268" t="s">
+        <v>58</v>
+      </c>
+      <c r="AD268" t="s">
+        <v>543</v>
+      </c>
+      <c r="AE268" t="s">
+        <v>58</v>
+      </c>
+      <c r="AF268" t="s">
+        <v>63</v>
+      </c>
+      <c r="AG268">
+        <v>-54</v>
+      </c>
+      <c r="AH268">
+        <v>0</v>
+      </c>
+      <c r="AI268">
+        <v>0</v>
+      </c>
+      <c r="AJ268" t="s">
+        <v>64</v>
+      </c>
+      <c r="AK268" t="s">
+        <v>65</v>
+      </c>
+      <c r="AL268" t="s">
+        <v>66</v>
+      </c>
+      <c r="AM268">
+        <v>971867</v>
+      </c>
+      <c r="AN268">
+        <v>134874</v>
+      </c>
+      <c r="AS268" t="s">
+        <v>85</v>
+      </c>
+      <c r="AT268" t="s">
+        <v>1230</v>
+      </c>
+      <c r="AU268" t="s">
+        <v>87</v>
+      </c>
+      <c r="AV268" t="s">
+        <v>1231</v>
+      </c>
+    </row>
+    <row r="269" spans="1:48" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A269" t="s">
+        <v>48</v>
+      </c>
+      <c r="B269" t="s">
+        <v>559</v>
+      </c>
+      <c r="C269" t="s">
+        <v>737</v>
+      </c>
+      <c r="D269" t="s">
+        <v>1232</v>
+      </c>
+      <c r="E269" t="s">
+        <v>1233</v>
+      </c>
+      <c r="F269" t="s">
+        <v>53</v>
+      </c>
+      <c r="G269" t="s">
+        <v>119</v>
+      </c>
+      <c r="H269" t="s">
+        <v>55</v>
+      </c>
+      <c r="I269">
+        <v>2841</v>
+      </c>
+      <c r="J269" t="s">
+        <v>56</v>
+      </c>
+      <c r="K269">
+        <v>35000</v>
+      </c>
+      <c r="L269">
+        <v>35000</v>
+      </c>
+      <c r="M269">
+        <v>36</v>
+      </c>
+      <c r="N269">
+        <v>5</v>
+      </c>
+      <c r="O269" t="s">
+        <v>1178</v>
+      </c>
+      <c r="P269">
+        <v>35000</v>
+      </c>
+      <c r="Q269">
+        <v>35000</v>
+      </c>
+      <c r="R269" t="s">
+        <v>58</v>
+      </c>
+      <c r="S269">
+        <v>34</v>
+      </c>
+      <c r="T269">
+        <v>2</v>
+      </c>
+      <c r="U269">
+        <v>1</v>
+      </c>
+      <c r="V269">
+        <v>2</v>
+      </c>
+      <c r="W269" t="s">
+        <v>59</v>
+      </c>
+      <c r="X269" t="s">
+        <v>157</v>
+      </c>
+      <c r="Y269" t="s">
+        <v>61</v>
+      </c>
+      <c r="Z269" t="s">
+        <v>1234</v>
+      </c>
+      <c r="AA269" t="s">
+        <v>1234</v>
+      </c>
+      <c r="AB269" t="s">
+        <v>58</v>
+      </c>
+      <c r="AD269" t="s">
+        <v>187</v>
+      </c>
+      <c r="AE269" t="s">
+        <v>58</v>
+      </c>
+      <c r="AF269" t="s">
+        <v>63</v>
+      </c>
+      <c r="AG269">
+        <v>-29</v>
+      </c>
+      <c r="AH269">
+        <v>0</v>
+      </c>
+      <c r="AI269">
+        <v>0</v>
+      </c>
+      <c r="AJ269" t="s">
+        <v>64</v>
+      </c>
+      <c r="AK269" t="s">
+        <v>65</v>
+      </c>
+      <c r="AL269" t="s">
+        <v>66</v>
+      </c>
+      <c r="AM269">
+        <v>971869</v>
+      </c>
+      <c r="AN269">
+        <v>134884</v>
+      </c>
+      <c r="AS269" t="s">
+        <v>202</v>
+      </c>
+      <c r="AT269" t="s">
+        <v>1235</v>
+      </c>
+      <c r="AV269" t="s">
+        <v>1236</v>
+      </c>
+    </row>
+    <row r="270" spans="1:48" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A270" t="s">
+        <v>48</v>
+      </c>
+      <c r="B270" t="s">
+        <v>49</v>
+      </c>
+      <c r="C270" t="s">
+        <v>1237</v>
+      </c>
+      <c r="D270" t="s">
+        <v>1238</v>
+      </c>
+      <c r="E270" t="s">
+        <v>1239</v>
+      </c>
+      <c r="F270" t="s">
+        <v>53</v>
+      </c>
+      <c r="G270" t="s">
+        <v>54</v>
+      </c>
+      <c r="H270" t="s">
+        <v>55</v>
+      </c>
+      <c r="I270">
+        <v>2660</v>
+      </c>
+      <c r="J270" t="s">
+        <v>56</v>
+      </c>
+      <c r="K270">
+        <v>30000</v>
+      </c>
+      <c r="L270">
+        <v>30000</v>
+      </c>
+      <c r="M270">
+        <v>60</v>
+      </c>
+      <c r="N270">
+        <v>5</v>
+      </c>
+      <c r="O270" t="s">
+        <v>1178</v>
+      </c>
+      <c r="P270">
+        <v>30000</v>
+      </c>
+      <c r="Q270">
+        <v>30000</v>
+      </c>
+      <c r="R270" t="s">
+        <v>58</v>
+      </c>
+      <c r="S270">
+        <v>55</v>
+      </c>
+      <c r="T270">
+        <v>5</v>
+      </c>
+      <c r="U270">
+        <v>1</v>
+      </c>
+      <c r="V270">
+        <v>5</v>
+      </c>
+      <c r="W270" t="s">
+        <v>59</v>
+      </c>
+      <c r="X270" t="s">
+        <v>60</v>
+      </c>
+      <c r="Y270" t="s">
+        <v>61</v>
+      </c>
+      <c r="Z270" t="s">
+        <v>62</v>
+      </c>
+      <c r="AA270" t="s">
+        <v>62</v>
+      </c>
+      <c r="AB270" t="s">
+        <v>58</v>
+      </c>
+      <c r="AD270" t="s">
+        <v>62</v>
+      </c>
+      <c r="AE270" t="s">
+        <v>58</v>
+      </c>
+      <c r="AF270" t="s">
+        <v>63</v>
+      </c>
+      <c r="AG270">
+        <v>-29</v>
+      </c>
+      <c r="AH270">
+        <v>0</v>
+      </c>
+      <c r="AI270">
+        <v>0</v>
+      </c>
+      <c r="AJ270" t="s">
+        <v>64</v>
+      </c>
+      <c r="AK270" t="s">
+        <v>65</v>
+      </c>
+      <c r="AL270" t="s">
+        <v>66</v>
+      </c>
+      <c r="AM270">
+        <v>971870</v>
+      </c>
+      <c r="AN270">
+        <v>134834</v>
+      </c>
+      <c r="AS270" t="s">
+        <v>85</v>
+      </c>
+      <c r="AT270" t="s">
+        <v>1240</v>
+      </c>
+      <c r="AU270" t="s">
+        <v>1241</v>
+      </c>
+      <c r="AV270" t="s">
+        <v>1241</v>
+      </c>
+    </row>
+    <row r="271" spans="1:48" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A271" t="s">
+        <v>48</v>
+      </c>
+      <c r="B271" t="s">
+        <v>1242</v>
+      </c>
+      <c r="C271" t="s">
+        <v>782</v>
+      </c>
+      <c r="D271" t="s">
+        <v>1243</v>
+      </c>
+      <c r="E271" t="s">
+        <v>1244</v>
+      </c>
+      <c r="F271" t="s">
+        <v>53</v>
+      </c>
+      <c r="G271" t="s">
+        <v>311</v>
+      </c>
+      <c r="H271" t="s">
+        <v>55</v>
+      </c>
+      <c r="I271">
+        <v>2332</v>
+      </c>
+      <c r="J271" t="s">
+        <v>56</v>
+      </c>
+      <c r="K271">
+        <v>25000</v>
+      </c>
+      <c r="L271">
+        <v>25000</v>
+      </c>
+      <c r="M271">
+        <v>60</v>
+      </c>
+      <c r="N271">
+        <v>5</v>
+      </c>
+      <c r="O271" t="s">
+        <v>1178</v>
+      </c>
+      <c r="P271">
+        <v>25000</v>
+      </c>
+      <c r="Q271">
+        <v>25000</v>
+      </c>
+      <c r="R271" t="s">
+        <v>58</v>
+      </c>
+      <c r="S271">
+        <v>55</v>
+      </c>
+      <c r="T271">
+        <v>5</v>
+      </c>
+      <c r="U271">
+        <v>1</v>
+      </c>
+      <c r="V271">
+        <v>5</v>
+      </c>
+      <c r="W271" t="s">
+        <v>59</v>
+      </c>
+      <c r="X271" t="s">
+        <v>210</v>
+      </c>
+      <c r="Y271" t="s">
+        <v>61</v>
+      </c>
+      <c r="Z271" t="s">
+        <v>1245</v>
+      </c>
+      <c r="AA271" t="s">
+        <v>1245</v>
+      </c>
+      <c r="AB271" t="s">
+        <v>58</v>
+      </c>
+      <c r="AD271" t="s">
+        <v>1246</v>
+      </c>
+      <c r="AE271" t="s">
+        <v>58</v>
+      </c>
+      <c r="AF271" t="s">
+        <v>1247</v>
+      </c>
+      <c r="AG271">
+        <v>2</v>
+      </c>
+      <c r="AH271">
+        <v>0</v>
+      </c>
+      <c r="AI271">
+        <v>0</v>
+      </c>
+      <c r="AJ271" t="s">
+        <v>64</v>
+      </c>
+      <c r="AK271" t="s">
+        <v>65</v>
+      </c>
+      <c r="AL271" t="s">
+        <v>66</v>
+      </c>
+      <c r="AM271">
+        <v>971880</v>
+      </c>
+      <c r="AN271">
+        <v>134735</v>
+      </c>
+      <c r="AS271" t="s">
+        <v>85</v>
+      </c>
+      <c r="AT271" t="s">
+        <v>1248</v>
+      </c>
+      <c r="AU271" t="s">
+        <v>87</v>
+      </c>
+      <c r="AV271" t="s">
+        <v>1249</v>
+      </c>
+    </row>
+    <row r="272" spans="1:48" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A272" t="s">
+        <v>48</v>
+      </c>
+      <c r="B272" t="s">
+        <v>676</v>
+      </c>
+      <c r="C272" t="s">
+        <v>279</v>
+      </c>
+      <c r="D272" t="s">
+        <v>1250</v>
+      </c>
+      <c r="E272" t="s">
+        <v>1251</v>
+      </c>
+      <c r="F272" t="s">
+        <v>53</v>
+      </c>
+      <c r="G272" t="s">
+        <v>119</v>
+      </c>
+      <c r="H272" t="s">
+        <v>75</v>
+      </c>
+      <c r="I272">
+        <v>1571</v>
+      </c>
+      <c r="J272" t="s">
+        <v>56</v>
+      </c>
+      <c r="K272">
+        <v>33750</v>
+      </c>
+      <c r="L272">
+        <v>33750</v>
+      </c>
+      <c r="M272">
+        <v>48</v>
+      </c>
+      <c r="N272">
+        <v>10</v>
+      </c>
+      <c r="O272" t="s">
+        <v>1178</v>
+      </c>
+      <c r="P272">
+        <v>33500</v>
+      </c>
+      <c r="Q272">
+        <v>33500</v>
+      </c>
+      <c r="R272" t="s">
+        <v>58</v>
+      </c>
+      <c r="S272">
+        <v>39</v>
+      </c>
+      <c r="T272">
+        <v>9</v>
+      </c>
+      <c r="U272">
+        <v>1</v>
+      </c>
+      <c r="V272">
+        <v>9</v>
+      </c>
+      <c r="W272" t="s">
+        <v>59</v>
+      </c>
+      <c r="X272" t="s">
+        <v>210</v>
+      </c>
+      <c r="Y272" t="s">
+        <v>61</v>
+      </c>
+      <c r="Z272" t="s">
+        <v>199</v>
+      </c>
+      <c r="AA272" t="s">
+        <v>199</v>
+      </c>
+      <c r="AB272" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC272" t="s">
+        <v>129</v>
+      </c>
+      <c r="AD272" t="s">
+        <v>200</v>
+      </c>
+      <c r="AE272" t="s">
+        <v>58</v>
+      </c>
+      <c r="AF272" t="s">
+        <v>63</v>
+      </c>
+      <c r="AG272">
+        <v>-95</v>
+      </c>
+      <c r="AH272">
+        <v>30</v>
+      </c>
+      <c r="AI272">
+        <v>0</v>
+      </c>
+      <c r="AJ272" t="s">
+        <v>64</v>
+      </c>
+      <c r="AK272" t="s">
+        <v>65</v>
+      </c>
+      <c r="AL272" t="s">
+        <v>66</v>
+      </c>
+      <c r="AM272">
+        <v>971882</v>
+      </c>
+      <c r="AN272">
+        <v>134428</v>
+      </c>
+      <c r="AS272" t="s">
+        <v>77</v>
+      </c>
+      <c r="AT272" t="s">
+        <v>1252</v>
+      </c>
+      <c r="AU272" t="s">
+        <v>1253</v>
+      </c>
+      <c r="AV272" t="s">
+        <v>1254</v>
+      </c>
+    </row>
+    <row r="273" spans="1:48" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A273" t="s">
+        <v>48</v>
+      </c>
+      <c r="B273" t="s">
+        <v>1255</v>
+      </c>
+      <c r="C273" t="s">
+        <v>1256</v>
+      </c>
+      <c r="D273" t="s">
+        <v>1257</v>
+      </c>
+      <c r="E273" t="s">
+        <v>1258</v>
+      </c>
+      <c r="F273" t="s">
+        <v>53</v>
+      </c>
+      <c r="G273" t="s">
+        <v>882</v>
+      </c>
+      <c r="H273" t="s">
+        <v>104</v>
+      </c>
+      <c r="I273">
+        <v>149</v>
+      </c>
+      <c r="J273" t="s">
+        <v>56</v>
+      </c>
+      <c r="K273">
+        <v>28000</v>
+      </c>
+      <c r="L273">
+        <v>28000</v>
+      </c>
+      <c r="M273">
+        <v>36</v>
+      </c>
+      <c r="N273">
+        <v>5</v>
+      </c>
+      <c r="O273" t="s">
+        <v>1178</v>
+      </c>
+      <c r="P273">
+        <v>28000</v>
+      </c>
+      <c r="Q273">
+        <v>28000</v>
+      </c>
+      <c r="R273" t="s">
+        <v>58</v>
+      </c>
+      <c r="S273">
+        <v>18</v>
+      </c>
+      <c r="T273">
+        <v>18</v>
+      </c>
+      <c r="U273">
+        <v>1</v>
+      </c>
+      <c r="V273">
+        <v>18</v>
+      </c>
+      <c r="W273" t="s">
+        <v>7</v>
+      </c>
+      <c r="X273" t="s">
+        <v>240</v>
+      </c>
+      <c r="Y273" t="s">
+        <v>61</v>
+      </c>
+      <c r="Z273" t="s">
+        <v>550</v>
+      </c>
+      <c r="AA273" t="s">
+        <v>550</v>
+      </c>
+      <c r="AB273" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC273" t="s">
+        <v>95</v>
+      </c>
+      <c r="AD273" t="s">
+        <v>543</v>
+      </c>
+      <c r="AE273" t="s">
+        <v>58</v>
+      </c>
+      <c r="AF273" t="s">
+        <v>409</v>
+      </c>
+      <c r="AG273">
+        <v>-29</v>
+      </c>
+      <c r="AH273">
+        <v>0</v>
+      </c>
+      <c r="AI273">
+        <v>0</v>
+      </c>
+      <c r="AJ273" t="s">
+        <v>64</v>
+      </c>
+      <c r="AK273" t="s">
+        <v>65</v>
+      </c>
+      <c r="AL273" t="s">
+        <v>66</v>
+      </c>
+      <c r="AM273">
+        <v>971884</v>
+      </c>
+      <c r="AN273">
+        <v>133305</v>
+      </c>
+      <c r="AS273" t="s">
+        <v>202</v>
+      </c>
+      <c r="AT273" t="s">
+        <v>1259</v>
+      </c>
+      <c r="AU273" t="s">
+        <v>1260</v>
+      </c>
+      <c r="AV273" t="s">
+        <v>1260</v>
+      </c>
+    </row>
+    <row r="274" spans="1:48" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A274" t="s">
+        <v>48</v>
+      </c>
+      <c r="B274" t="s">
+        <v>1255</v>
+      </c>
+      <c r="C274" t="s">
+        <v>1256</v>
+      </c>
+      <c r="D274" t="s">
+        <v>1261</v>
+      </c>
+      <c r="E274" t="s">
+        <v>1262</v>
+      </c>
+      <c r="F274" t="s">
+        <v>53</v>
+      </c>
+      <c r="G274" t="s">
+        <v>882</v>
+      </c>
+      <c r="H274" t="s">
+        <v>104</v>
+      </c>
+      <c r="I274">
+        <v>147</v>
+      </c>
+      <c r="J274" t="s">
+        <v>56</v>
+      </c>
+      <c r="K274">
+        <v>36000</v>
+      </c>
+      <c r="L274">
+        <v>36000</v>
+      </c>
+      <c r="M274">
+        <v>36</v>
+      </c>
+      <c r="N274">
+        <v>5</v>
+      </c>
+      <c r="O274" t="s">
+        <v>1178</v>
+      </c>
+      <c r="P274">
+        <v>36000</v>
+      </c>
+      <c r="Q274">
+        <v>36000</v>
+      </c>
+      <c r="R274" t="s">
+        <v>58</v>
+      </c>
+      <c r="S274">
+        <v>18</v>
+      </c>
+      <c r="T274">
+        <v>18</v>
+      </c>
+      <c r="U274">
+        <v>1</v>
+      </c>
+      <c r="V274">
+        <v>18</v>
+      </c>
+      <c r="W274" t="s">
+        <v>7</v>
+      </c>
+      <c r="X274" t="s">
+        <v>240</v>
+      </c>
+      <c r="Y274" t="s">
+        <v>61</v>
+      </c>
+      <c r="Z274" t="s">
+        <v>550</v>
+      </c>
+      <c r="AA274" t="s">
+        <v>550</v>
+      </c>
+      <c r="AB274" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC274" t="s">
+        <v>95</v>
+      </c>
+      <c r="AD274" t="s">
+        <v>543</v>
+      </c>
+      <c r="AE274" t="s">
+        <v>58</v>
+      </c>
+      <c r="AF274" t="s">
+        <v>409</v>
+      </c>
+      <c r="AG274">
+        <v>-29</v>
+      </c>
+      <c r="AH274">
+        <v>0</v>
+      </c>
+      <c r="AI274">
+        <v>0</v>
+      </c>
+      <c r="AJ274" t="s">
+        <v>64</v>
+      </c>
+      <c r="AK274" t="s">
+        <v>65</v>
+      </c>
+      <c r="AL274" t="s">
+        <v>66</v>
+      </c>
+      <c r="AM274">
+        <v>971886</v>
+      </c>
+      <c r="AN274">
+        <v>133288</v>
+      </c>
+      <c r="AS274" t="s">
+        <v>225</v>
+      </c>
+      <c r="AT274" t="s">
+        <v>1263</v>
+      </c>
+      <c r="AU274" t="s">
+        <v>1264</v>
+      </c>
+      <c r="AV274" t="s">
+        <v>1264</v>
+      </c>
+    </row>
+    <row r="275" spans="1:48" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A275" t="s">
+        <v>48</v>
+      </c>
+      <c r="B275" t="s">
+        <v>1265</v>
+      </c>
+      <c r="C275" t="s">
+        <v>723</v>
+      </c>
+      <c r="D275" t="s">
+        <v>1266</v>
+      </c>
+      <c r="E275" t="s">
+        <v>1267</v>
+      </c>
+      <c r="F275" t="s">
+        <v>53</v>
+      </c>
+      <c r="G275" t="s">
+        <v>452</v>
+      </c>
+      <c r="H275" t="s">
+        <v>55</v>
+      </c>
+      <c r="I275">
+        <v>2415</v>
+      </c>
+      <c r="J275" t="s">
+        <v>56</v>
+      </c>
+      <c r="K275">
+        <v>42500</v>
+      </c>
+      <c r="L275">
+        <v>42500</v>
+      </c>
+      <c r="M275">
+        <v>36</v>
+      </c>
+      <c r="N275">
+        <v>1</v>
+      </c>
+      <c r="O275" t="s">
+        <v>1178</v>
+      </c>
+      <c r="P275">
+        <v>42500</v>
+      </c>
+      <c r="Q275">
+        <v>42500</v>
+      </c>
+      <c r="R275" t="s">
+        <v>58</v>
+      </c>
+      <c r="S275">
+        <v>29</v>
+      </c>
+      <c r="T275">
+        <v>7</v>
+      </c>
+      <c r="U275">
+        <v>1</v>
+      </c>
+      <c r="V275">
+        <v>7</v>
+      </c>
+      <c r="W275" t="s">
+        <v>59</v>
+      </c>
+      <c r="X275" t="s">
+        <v>240</v>
+      </c>
+      <c r="Y275" t="s">
+        <v>61</v>
+      </c>
+      <c r="Z275" t="s">
+        <v>550</v>
+      </c>
+      <c r="AA275" t="s">
+        <v>550</v>
+      </c>
+      <c r="AB275" t="s">
+        <v>58</v>
+      </c>
+      <c r="AD275" t="s">
+        <v>543</v>
+      </c>
+      <c r="AE275" t="s">
+        <v>58</v>
+      </c>
+      <c r="AF275" t="s">
+        <v>63</v>
+      </c>
+      <c r="AG275">
+        <v>-86</v>
+      </c>
+      <c r="AH275">
+        <v>0</v>
+      </c>
+      <c r="AI275">
+        <v>0</v>
+      </c>
+      <c r="AJ275" t="s">
+        <v>64</v>
+      </c>
+      <c r="AK275" t="s">
+        <v>65</v>
+      </c>
+      <c r="AL275" t="s">
+        <v>66</v>
+      </c>
+      <c r="AM275">
+        <v>971888</v>
+      </c>
+      <c r="AN275">
+        <v>134756</v>
+      </c>
+      <c r="AS275" t="s">
+        <v>202</v>
+      </c>
+      <c r="AT275" t="s">
+        <v>1268</v>
+      </c>
+      <c r="AU275" t="s">
+        <v>87</v>
+      </c>
+      <c r="AV275" t="s">
+        <v>1269</v>
+      </c>
+    </row>
+    <row r="276" spans="1:48" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A276" t="s">
+        <v>48</v>
+      </c>
+      <c r="B276" t="s">
+        <v>1270</v>
+      </c>
+      <c r="C276" t="s">
+        <v>1271</v>
+      </c>
+      <c r="D276" t="s">
+        <v>1272</v>
+      </c>
+      <c r="E276" t="s">
+        <v>1273</v>
+      </c>
+      <c r="F276" t="s">
+        <v>53</v>
+      </c>
+      <c r="G276" t="s">
+        <v>452</v>
+      </c>
+      <c r="H276" t="s">
+        <v>55</v>
+      </c>
+      <c r="I276">
+        <v>3998</v>
+      </c>
+      <c r="J276" t="s">
+        <v>56</v>
+      </c>
+      <c r="K276">
+        <v>35750</v>
+      </c>
+      <c r="L276">
+        <v>35750</v>
+      </c>
+      <c r="M276">
+        <v>36</v>
+      </c>
+      <c r="N276">
+        <v>9</v>
+      </c>
+      <c r="O276" t="s">
+        <v>1178</v>
+      </c>
+      <c r="P276">
+        <v>35750</v>
+      </c>
+      <c r="Q276">
+        <v>35750</v>
+      </c>
+      <c r="R276" t="s">
+        <v>58</v>
+      </c>
+      <c r="S276">
+        <v>35</v>
+      </c>
+      <c r="T276">
+        <v>2</v>
+      </c>
+      <c r="U276">
+        <v>1</v>
+      </c>
+      <c r="V276">
+        <v>1</v>
+      </c>
+      <c r="W276" t="s">
+        <v>59</v>
+      </c>
+      <c r="X276" t="s">
+        <v>240</v>
+      </c>
+      <c r="Y276" t="s">
+        <v>61</v>
+      </c>
+      <c r="Z276" t="s">
+        <v>550</v>
+      </c>
+      <c r="AA276" t="s">
+        <v>550</v>
+      </c>
+      <c r="AB276" t="s">
+        <v>58</v>
+      </c>
+      <c r="AD276" t="s">
+        <v>543</v>
+      </c>
+      <c r="AE276" t="s">
+        <v>58</v>
+      </c>
+      <c r="AF276" t="s">
+        <v>63</v>
+      </c>
+      <c r="AG276">
+        <v>-33</v>
+      </c>
+      <c r="AH276">
+        <v>0</v>
+      </c>
+      <c r="AI276">
+        <v>0</v>
+      </c>
+      <c r="AJ276" t="s">
+        <v>64</v>
+      </c>
+      <c r="AK276" t="s">
+        <v>65</v>
+      </c>
+      <c r="AL276" t="s">
+        <v>66</v>
+      </c>
+      <c r="AM276">
+        <v>971890</v>
+      </c>
+      <c r="AN276">
+        <v>135208</v>
+      </c>
+      <c r="AS276" t="s">
+        <v>202</v>
+      </c>
+      <c r="AT276" t="s">
+        <v>1274</v>
+      </c>
+      <c r="AU276" t="s">
+        <v>1275</v>
+      </c>
+      <c r="AV276" t="s">
+        <v>1276</v>
+      </c>
+    </row>
+    <row r="277" spans="1:48" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A277" t="s">
+        <v>48</v>
+      </c>
+      <c r="B277" t="s">
+        <v>1270</v>
+      </c>
+      <c r="C277" t="s">
+        <v>1271</v>
+      </c>
+      <c r="D277" t="s">
+        <v>1272</v>
+      </c>
+      <c r="E277" t="s">
+        <v>1273</v>
+      </c>
+      <c r="F277" t="s">
+        <v>53</v>
+      </c>
+      <c r="G277" t="s">
+        <v>452</v>
+      </c>
+      <c r="H277" t="s">
+        <v>55</v>
+      </c>
+      <c r="I277">
+        <v>3998</v>
+      </c>
+      <c r="J277" t="s">
+        <v>56</v>
+      </c>
+      <c r="K277">
+        <v>35750</v>
+      </c>
+      <c r="L277">
+        <v>35750</v>
+      </c>
+      <c r="M277">
+        <v>36</v>
+      </c>
+      <c r="N277">
+        <v>9</v>
+      </c>
+      <c r="O277" t="s">
+        <v>1178</v>
+      </c>
+      <c r="P277">
+        <v>2000</v>
+      </c>
+      <c r="Q277">
+        <v>2000</v>
+      </c>
+      <c r="R277" t="s">
+        <v>58</v>
+      </c>
+      <c r="S277">
+        <v>35</v>
+      </c>
+      <c r="T277">
+        <v>2</v>
+      </c>
+      <c r="U277">
+        <v>1</v>
+      </c>
+      <c r="V277">
+        <v>2</v>
+      </c>
+      <c r="W277" t="s">
+        <v>59</v>
+      </c>
+      <c r="X277" t="s">
+        <v>240</v>
+      </c>
+      <c r="Y277" t="s">
+        <v>61</v>
+      </c>
+      <c r="Z277" t="s">
+        <v>550</v>
+      </c>
+      <c r="AA277" t="s">
+        <v>550</v>
+      </c>
+      <c r="AB277" t="s">
+        <v>58</v>
+      </c>
+      <c r="AD277" t="s">
+        <v>543</v>
+      </c>
+      <c r="AE277" t="s">
+        <v>58</v>
+      </c>
+      <c r="AF277" t="s">
+        <v>63</v>
+      </c>
+      <c r="AG277">
+        <v>-33</v>
+      </c>
+      <c r="AH277">
+        <v>0</v>
+      </c>
+      <c r="AI277">
+        <v>0</v>
+      </c>
+      <c r="AJ277" t="s">
+        <v>64</v>
+      </c>
+      <c r="AK277" t="s">
+        <v>65</v>
+      </c>
+      <c r="AL277" t="s">
+        <v>66</v>
+      </c>
+      <c r="AM277">
+        <v>971890</v>
+      </c>
+      <c r="AN277">
+        <v>135208</v>
+      </c>
+      <c r="AS277" t="s">
+        <v>202</v>
+      </c>
+      <c r="AT277" t="s">
+        <v>1274</v>
+      </c>
+      <c r="AU277" t="s">
+        <v>1275</v>
+      </c>
+      <c r="AV277" t="s">
+        <v>1276</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:AV258" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:AV277" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -38258,13 +41023,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D7E3B6AB-27EB-4F9F-8365-4BF40A6CCD02}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9C59DCED-5F63-43D6-B8D8-81E621B5A6A1}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DDDB2C88-4B0E-427D-AA90-F20137981B9F}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2E8098D5-7410-4870-BAC7-6609AEB8FB6C}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{791BBE6B-688E-4179-B895-34F2EAA5A859}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2424B923-134C-4B06-AB06-0A75CC9D5A01}"/>
 </file>
</xml_diff>